<commit_message>
Respaldo automático: 2026-10-14 09:30
</commit_message>
<xml_diff>
--- a/2026-2/ListadoEstudiantes.xlsx
+++ b/2026-2/ListadoEstudiantes.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/unicordoba/Documents/Cursos/Computacional/2026-2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{549791D7-575F-274A-89A1-195567AC6820}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC373DAD-26F5-A542-ADDF-497BA85DF223}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="14400" windowHeight="16180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$C$1:$C$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$G$1:$G$47</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="150">
   <si>
     <t>Nombre</t>
   </si>
@@ -275,15 +275,6 @@
     <t>ferneydavidmarzola@gmail.com</t>
   </si>
   <si>
-    <t>MARIO ALFONSO</t>
-  </si>
-  <si>
-    <t>MORALES RIVERA</t>
-  </si>
-  <si>
-    <t>mamorales@correo.unicordoba.edu.co</t>
-  </si>
-  <si>
     <t>NAYELIS</t>
   </si>
   <si>
@@ -483,6 +474,18 @@
   </si>
   <si>
     <t>Septiembre 4 de 2026</t>
+  </si>
+  <si>
+    <t>Septiembre 11 de 2026</t>
+  </si>
+  <si>
+    <t>Septiembre 16 de 2026</t>
+  </si>
+  <si>
+    <t>Septiembre 18 de 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total fallas </t>
   </si>
 </sst>
 </file>
@@ -859,20 +862,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:P47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="10" width="22.6640625" customWidth="1"/>
+    <col min="2" max="2" width="19.1640625" customWidth="1"/>
+    <col min="3" max="3" width="9.1640625" customWidth="1"/>
+    <col min="4" max="14" width="22.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>149</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>148</v>
@@ -883,26 +890,35 @@
       <c r="F1" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>144</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>142</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="O1" t="s">
         <v>2</v>
       </c>
-      <c r="L1" t="s">
+      <c r="P1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -910,10 +926,11 @@
         <v>5</v>
       </c>
       <c r="C2">
+        <f>11-SUM(D2:N2)</f>
         <v>1</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -933,11 +950,23 @@
       <c r="J2">
         <v>1</v>
       </c>
-      <c r="K2" t="s">
+      <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="L2">
+        <v>1</v>
+      </c>
+      <c r="M2">
+        <v>1</v>
+      </c>
+      <c r="N2">
+        <v>1</v>
+      </c>
+      <c r="O2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -945,6 +974,7 @@
         <v>8</v>
       </c>
       <c r="C3">
+        <f t="shared" ref="C3:C46" si="0">11-SUM(D3:N3)</f>
         <v>1</v>
       </c>
       <c r="D3">
@@ -954,7 +984,7 @@
         <v>1</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G3">
         <v>1</v>
@@ -968,11 +998,23 @@
       <c r="J3">
         <v>1</v>
       </c>
-      <c r="K3" t="s">
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <v>1</v>
+      </c>
+      <c r="M3">
+        <v>1</v>
+      </c>
+      <c r="N3">
+        <v>1</v>
+      </c>
+      <c r="O3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -980,16 +1022,17 @@
         <v>11</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>2</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4">
         <v>1</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G4">
         <v>1</v>
@@ -1003,11 +1046,23 @@
       <c r="J4">
         <v>1</v>
       </c>
-      <c r="K4" t="s">
+      <c r="K4">
+        <v>1</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4">
+        <v>1</v>
+      </c>
+      <c r="N4">
+        <v>1</v>
+      </c>
+      <c r="O4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -1015,7 +1070,8 @@
         <v>14</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -1038,11 +1094,23 @@
       <c r="J5">
         <v>1</v>
       </c>
-      <c r="K5" t="s">
+      <c r="K5">
+        <v>1</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
+      <c r="M5">
+        <v>1</v>
+      </c>
+      <c r="N5">
+        <v>1</v>
+      </c>
+      <c r="O5" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -1050,7 +1118,8 @@
         <v>17</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -1073,11 +1142,23 @@
       <c r="J6">
         <v>1</v>
       </c>
-      <c r="K6" t="s">
+      <c r="K6">
+        <v>1</v>
+      </c>
+      <c r="L6">
+        <v>1</v>
+      </c>
+      <c r="M6">
+        <v>1</v>
+      </c>
+      <c r="N6">
+        <v>1</v>
+      </c>
+      <c r="O6" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -1085,19 +1166,20 @@
         <v>20</v>
       </c>
       <c r="C7">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>2</v>
       </c>
       <c r="D7">
         <v>1</v>
       </c>
       <c r="E7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F7">
         <v>1</v>
       </c>
       <c r="G7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H7">
         <v>1</v>
@@ -1108,11 +1190,23 @@
       <c r="J7">
         <v>1</v>
       </c>
-      <c r="K7" t="s">
+      <c r="K7">
+        <v>0</v>
+      </c>
+      <c r="L7">
+        <v>1</v>
+      </c>
+      <c r="M7">
+        <v>1</v>
+      </c>
+      <c r="N7">
+        <v>1</v>
+      </c>
+      <c r="O7" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>22</v>
       </c>
@@ -1120,7 +1214,8 @@
         <v>23</v>
       </c>
       <c r="C8">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -1143,11 +1238,23 @@
       <c r="J8">
         <v>1</v>
       </c>
-      <c r="K8" t="s">
+      <c r="K8">
+        <v>1</v>
+      </c>
+      <c r="L8">
+        <v>1</v>
+      </c>
+      <c r="M8">
+        <v>1</v>
+      </c>
+      <c r="N8">
+        <v>1</v>
+      </c>
+      <c r="O8" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>25</v>
       </c>
@@ -1155,7 +1262,8 @@
         <v>26</v>
       </c>
       <c r="C9">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -1178,11 +1286,23 @@
       <c r="J9">
         <v>1</v>
       </c>
-      <c r="K9" t="s">
+      <c r="K9">
+        <v>1</v>
+      </c>
+      <c r="L9">
+        <v>1</v>
+      </c>
+      <c r="M9">
+        <v>1</v>
+      </c>
+      <c r="N9">
+        <v>1</v>
+      </c>
+      <c r="O9" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>28</v>
       </c>
@@ -1190,7 +1310,8 @@
         <v>29</v>
       </c>
       <c r="C10">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>2</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -1202,10 +1323,10 @@
         <v>1</v>
       </c>
       <c r="G10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I10">
         <v>1</v>
@@ -1213,11 +1334,23 @@
       <c r="J10">
         <v>1</v>
       </c>
-      <c r="K10" t="s">
+      <c r="K10">
+        <v>0</v>
+      </c>
+      <c r="L10">
+        <v>0</v>
+      </c>
+      <c r="M10">
+        <v>1</v>
+      </c>
+      <c r="N10">
+        <v>1</v>
+      </c>
+      <c r="O10" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>31</v>
       </c>
@@ -1225,7 +1358,8 @@
         <v>32</v>
       </c>
       <c r="C11">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D11">
         <v>1</v>
@@ -1248,11 +1382,23 @@
       <c r="J11">
         <v>1</v>
       </c>
-      <c r="K11" t="s">
+      <c r="K11">
+        <v>1</v>
+      </c>
+      <c r="L11">
+        <v>1</v>
+      </c>
+      <c r="M11">
+        <v>1</v>
+      </c>
+      <c r="N11">
+        <v>1</v>
+      </c>
+      <c r="O11" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>34</v>
       </c>
@@ -1260,7 +1406,8 @@
         <v>35</v>
       </c>
       <c r="C12">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D12">
         <v>1</v>
@@ -1283,11 +1430,23 @@
       <c r="J12">
         <v>1</v>
       </c>
-      <c r="K12" t="s">
+      <c r="K12">
+        <v>1</v>
+      </c>
+      <c r="L12">
+        <v>1</v>
+      </c>
+      <c r="M12">
+        <v>1</v>
+      </c>
+      <c r="N12">
+        <v>1</v>
+      </c>
+      <c r="O12" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>37</v>
       </c>
@@ -1295,7 +1454,8 @@
         <v>38</v>
       </c>
       <c r="C13">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>3</v>
       </c>
       <c r="D13">
         <v>1</v>
@@ -1304,7 +1464,7 @@
         <v>1</v>
       </c>
       <c r="F13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G13">
         <v>1</v>
@@ -1313,16 +1473,28 @@
         <v>1</v>
       </c>
       <c r="I13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J13">
-        <v>0</v>
-      </c>
-      <c r="K13" t="s">
+        <v>1</v>
+      </c>
+      <c r="K13">
+        <v>1</v>
+      </c>
+      <c r="L13">
+        <v>1</v>
+      </c>
+      <c r="M13">
+        <v>0</v>
+      </c>
+      <c r="N13">
+        <v>0</v>
+      </c>
+      <c r="O13" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>40</v>
       </c>
@@ -1330,7 +1502,8 @@
         <v>41</v>
       </c>
       <c r="C14">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D14">
         <v>1</v>
@@ -1353,11 +1526,23 @@
       <c r="J14">
         <v>1</v>
       </c>
-      <c r="K14" t="s">
+      <c r="K14">
+        <v>1</v>
+      </c>
+      <c r="L14">
+        <v>1</v>
+      </c>
+      <c r="M14">
+        <v>1</v>
+      </c>
+      <c r="N14">
+        <v>1</v>
+      </c>
+      <c r="O14" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>43</v>
       </c>
@@ -1365,7 +1550,8 @@
         <v>44</v>
       </c>
       <c r="C15">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D15">
         <v>1</v>
@@ -1388,11 +1574,23 @@
       <c r="J15">
         <v>1</v>
       </c>
-      <c r="K15" t="s">
+      <c r="K15">
+        <v>1</v>
+      </c>
+      <c r="L15">
+        <v>1</v>
+      </c>
+      <c r="M15">
+        <v>1</v>
+      </c>
+      <c r="N15">
+        <v>1</v>
+      </c>
+      <c r="O15" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>46</v>
       </c>
@@ -1400,7 +1598,8 @@
         <v>47</v>
       </c>
       <c r="C16">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D16">
         <v>1</v>
@@ -1423,11 +1622,23 @@
       <c r="J16">
         <v>1</v>
       </c>
-      <c r="K16" t="s">
+      <c r="K16">
+        <v>1</v>
+      </c>
+      <c r="L16">
+        <v>1</v>
+      </c>
+      <c r="M16">
+        <v>1</v>
+      </c>
+      <c r="N16">
+        <v>1</v>
+      </c>
+      <c r="O16" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>49</v>
       </c>
@@ -1435,7 +1646,8 @@
         <v>50</v>
       </c>
       <c r="C17">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D17">
         <v>1</v>
@@ -1458,11 +1670,23 @@
       <c r="J17">
         <v>1</v>
       </c>
-      <c r="K17" t="s">
+      <c r="K17">
+        <v>1</v>
+      </c>
+      <c r="L17">
+        <v>1</v>
+      </c>
+      <c r="M17">
+        <v>1</v>
+      </c>
+      <c r="N17">
+        <v>1</v>
+      </c>
+      <c r="O17" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>52</v>
       </c>
@@ -1470,7 +1694,8 @@
         <v>53</v>
       </c>
       <c r="C18">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D18">
         <v>1</v>
@@ -1493,11 +1718,23 @@
       <c r="J18">
         <v>1</v>
       </c>
-      <c r="K18" t="s">
+      <c r="K18">
+        <v>1</v>
+      </c>
+      <c r="L18">
+        <v>1</v>
+      </c>
+      <c r="M18">
+        <v>1</v>
+      </c>
+      <c r="N18">
+        <v>1</v>
+      </c>
+      <c r="O18" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>55</v>
       </c>
@@ -1505,7 +1742,8 @@
         <v>56</v>
       </c>
       <c r="C19">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="D19">
         <v>1</v>
@@ -1517,7 +1755,7 @@
         <v>1</v>
       </c>
       <c r="G19">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H19">
         <v>1</v>
@@ -1528,11 +1766,23 @@
       <c r="J19">
         <v>1</v>
       </c>
-      <c r="K19" t="s">
+      <c r="K19">
+        <v>1</v>
+      </c>
+      <c r="L19">
+        <v>1</v>
+      </c>
+      <c r="M19">
+        <v>1</v>
+      </c>
+      <c r="N19">
+        <v>1</v>
+      </c>
+      <c r="O19" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>58</v>
       </c>
@@ -1540,7 +1790,8 @@
         <v>59</v>
       </c>
       <c r="C20">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D20">
         <v>1</v>
@@ -1563,11 +1814,23 @@
       <c r="J20">
         <v>1</v>
       </c>
-      <c r="K20" t="s">
+      <c r="K20">
+        <v>1</v>
+      </c>
+      <c r="L20">
+        <v>1</v>
+      </c>
+      <c r="M20">
+        <v>1</v>
+      </c>
+      <c r="N20">
+        <v>1</v>
+      </c>
+      <c r="O20" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>61</v>
       </c>
@@ -1575,7 +1838,8 @@
         <v>62</v>
       </c>
       <c r="C21">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D21">
         <v>1</v>
@@ -1598,11 +1862,23 @@
       <c r="J21">
         <v>1</v>
       </c>
-      <c r="K21" t="s">
+      <c r="K21">
+        <v>1</v>
+      </c>
+      <c r="L21">
+        <v>1</v>
+      </c>
+      <c r="M21">
+        <v>1</v>
+      </c>
+      <c r="N21">
+        <v>1</v>
+      </c>
+      <c r="O21" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>64</v>
       </c>
@@ -1610,7 +1886,8 @@
         <v>65</v>
       </c>
       <c r="C22">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D22">
         <v>1</v>
@@ -1633,11 +1910,23 @@
       <c r="J22">
         <v>1</v>
       </c>
-      <c r="K22" t="s">
+      <c r="K22">
+        <v>1</v>
+      </c>
+      <c r="L22">
+        <v>1</v>
+      </c>
+      <c r="M22">
+        <v>1</v>
+      </c>
+      <c r="N22">
+        <v>1</v>
+      </c>
+      <c r="O22" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>67</v>
       </c>
@@ -1645,7 +1934,8 @@
         <v>68</v>
       </c>
       <c r="C23">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D23">
         <v>1</v>
@@ -1668,11 +1958,23 @@
       <c r="J23">
         <v>1</v>
       </c>
-      <c r="K23" t="s">
+      <c r="K23">
+        <v>1</v>
+      </c>
+      <c r="L23">
+        <v>1</v>
+      </c>
+      <c r="M23">
+        <v>1</v>
+      </c>
+      <c r="N23">
+        <v>1</v>
+      </c>
+      <c r="O23" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>70</v>
       </c>
@@ -1680,7 +1982,8 @@
         <v>71</v>
       </c>
       <c r="C24">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>2</v>
       </c>
       <c r="D24">
         <v>1</v>
@@ -1695,19 +1998,31 @@
         <v>1</v>
       </c>
       <c r="H24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I24">
         <v>1</v>
       </c>
       <c r="J24">
-        <v>0</v>
-      </c>
-      <c r="K24" t="s">
+        <v>1</v>
+      </c>
+      <c r="K24">
+        <v>1</v>
+      </c>
+      <c r="L24">
+        <v>0</v>
+      </c>
+      <c r="M24">
+        <v>1</v>
+      </c>
+      <c r="N24">
+        <v>0</v>
+      </c>
+      <c r="O24" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>73</v>
       </c>
@@ -1715,6 +2030,7 @@
         <v>74</v>
       </c>
       <c r="C25">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="D25">
@@ -1733,16 +2049,28 @@
         <v>1</v>
       </c>
       <c r="I25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J25">
         <v>1</v>
       </c>
-      <c r="K25" t="s">
+      <c r="K25">
+        <v>1</v>
+      </c>
+      <c r="L25">
+        <v>1</v>
+      </c>
+      <c r="M25">
+        <v>0</v>
+      </c>
+      <c r="N25">
+        <v>1</v>
+      </c>
+      <c r="O25" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>76</v>
       </c>
@@ -1750,7 +2078,8 @@
         <v>77</v>
       </c>
       <c r="C26">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D26">
         <v>1</v>
@@ -1773,22 +2102,71 @@
       <c r="J26">
         <v>1</v>
       </c>
-      <c r="K26" t="s">
+      <c r="K26">
+        <v>1</v>
+      </c>
+      <c r="L26">
+        <v>1</v>
+      </c>
+      <c r="M26">
+        <v>1</v>
+      </c>
+      <c r="N26">
+        <v>1</v>
+      </c>
+      <c r="O26" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>79</v>
       </c>
       <c r="B27" t="s">
         <v>80</v>
       </c>
-      <c r="K27" t="s">
+      <c r="C27">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D27">
+        <v>1</v>
+      </c>
+      <c r="E27">
+        <v>1</v>
+      </c>
+      <c r="F27">
+        <v>1</v>
+      </c>
+      <c r="G27">
+        <v>1</v>
+      </c>
+      <c r="H27">
+        <v>1</v>
+      </c>
+      <c r="I27">
+        <v>1</v>
+      </c>
+      <c r="J27">
+        <v>1</v>
+      </c>
+      <c r="K27">
+        <v>1</v>
+      </c>
+      <c r="L27">
+        <v>1</v>
+      </c>
+      <c r="M27">
+        <v>1</v>
+      </c>
+      <c r="N27">
+        <v>1</v>
+      </c>
+      <c r="O27" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>82</v>
       </c>
@@ -1796,7 +2174,8 @@
         <v>83</v>
       </c>
       <c r="C28">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D28">
         <v>1</v>
@@ -1819,11 +2198,23 @@
       <c r="J28">
         <v>1</v>
       </c>
-      <c r="K28" t="s">
+      <c r="K28">
+        <v>1</v>
+      </c>
+      <c r="L28">
+        <v>1</v>
+      </c>
+      <c r="M28">
+        <v>1</v>
+      </c>
+      <c r="N28">
+        <v>1</v>
+      </c>
+      <c r="O28" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>85</v>
       </c>
@@ -1831,7 +2222,8 @@
         <v>86</v>
       </c>
       <c r="C29">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>3</v>
       </c>
       <c r="D29">
         <v>1</v>
@@ -1854,11 +2246,23 @@
       <c r="J29">
         <v>1</v>
       </c>
-      <c r="K29" t="s">
+      <c r="K29">
+        <v>0</v>
+      </c>
+      <c r="L29">
+        <v>1</v>
+      </c>
+      <c r="M29">
+        <v>0</v>
+      </c>
+      <c r="N29">
+        <v>0</v>
+      </c>
+      <c r="O29" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>88</v>
       </c>
@@ -1866,7 +2270,8 @@
         <v>89</v>
       </c>
       <c r="C30">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D30">
         <v>1</v>
@@ -1878,22 +2283,34 @@
         <v>1</v>
       </c>
       <c r="G30">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H30">
         <v>1</v>
       </c>
       <c r="I30">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J30">
-        <v>0</v>
-      </c>
-      <c r="K30" t="s">
+        <v>1</v>
+      </c>
+      <c r="K30">
+        <v>1</v>
+      </c>
+      <c r="L30">
+        <v>1</v>
+      </c>
+      <c r="M30">
+        <v>1</v>
+      </c>
+      <c r="N30">
+        <v>1</v>
+      </c>
+      <c r="O30" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>91</v>
       </c>
@@ -1901,7 +2318,8 @@
         <v>92</v>
       </c>
       <c r="C31">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>3</v>
       </c>
       <c r="D31">
         <v>1</v>
@@ -1910,25 +2328,37 @@
         <v>1</v>
       </c>
       <c r="F31">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G31">
         <v>1</v>
       </c>
       <c r="H31">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I31">
         <v>1</v>
       </c>
       <c r="J31">
-        <v>1</v>
-      </c>
-      <c r="K31" t="s">
+        <v>0</v>
+      </c>
+      <c r="K31">
+        <v>1</v>
+      </c>
+      <c r="L31">
+        <v>1</v>
+      </c>
+      <c r="M31">
+        <v>1</v>
+      </c>
+      <c r="N31">
+        <v>1</v>
+      </c>
+      <c r="O31" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>94</v>
       </c>
@@ -1936,16 +2366,17 @@
         <v>95</v>
       </c>
       <c r="C32">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D32">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E32">
         <v>1</v>
       </c>
       <c r="F32">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G32">
         <v>1</v>
@@ -1959,11 +2390,23 @@
       <c r="J32">
         <v>1</v>
       </c>
-      <c r="K32" t="s">
+      <c r="K32">
+        <v>1</v>
+      </c>
+      <c r="L32">
+        <v>1</v>
+      </c>
+      <c r="M32">
+        <v>1</v>
+      </c>
+      <c r="N32">
+        <v>1</v>
+      </c>
+      <c r="O32" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>97</v>
       </c>
@@ -1971,6 +2414,7 @@
         <v>98</v>
       </c>
       <c r="C33">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="D33">
@@ -1994,11 +2438,23 @@
       <c r="J33">
         <v>1</v>
       </c>
-      <c r="K33" t="s">
+      <c r="K33">
+        <v>0</v>
+      </c>
+      <c r="L33">
+        <v>1</v>
+      </c>
+      <c r="M33">
+        <v>1</v>
+      </c>
+      <c r="N33">
+        <v>1</v>
+      </c>
+      <c r="O33" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>100</v>
       </c>
@@ -2006,7 +2462,8 @@
         <v>101</v>
       </c>
       <c r="C34">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D34">
         <v>1</v>
@@ -2018,7 +2475,7 @@
         <v>1</v>
       </c>
       <c r="G34">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H34">
         <v>1</v>
@@ -2029,11 +2486,23 @@
       <c r="J34">
         <v>1</v>
       </c>
-      <c r="K34" t="s">
+      <c r="K34">
+        <v>1</v>
+      </c>
+      <c r="L34">
+        <v>1</v>
+      </c>
+      <c r="M34">
+        <v>1</v>
+      </c>
+      <c r="N34">
+        <v>1</v>
+      </c>
+      <c r="O34" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>103</v>
       </c>
@@ -2041,7 +2510,8 @@
         <v>104</v>
       </c>
       <c r="C35">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>2</v>
       </c>
       <c r="D35">
         <v>1</v>
@@ -2050,7 +2520,7 @@
         <v>1</v>
       </c>
       <c r="F35">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G35">
         <v>1</v>
@@ -2064,11 +2534,23 @@
       <c r="J35">
         <v>1</v>
       </c>
-      <c r="K35" t="s">
+      <c r="K35">
+        <v>1</v>
+      </c>
+      <c r="L35">
+        <v>0</v>
+      </c>
+      <c r="M35">
+        <v>1</v>
+      </c>
+      <c r="N35">
+        <v>1</v>
+      </c>
+      <c r="O35" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>106</v>
       </c>
@@ -2076,7 +2558,8 @@
         <v>107</v>
       </c>
       <c r="C36">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D36">
         <v>1</v>
@@ -2091,7 +2574,7 @@
         <v>1</v>
       </c>
       <c r="H36">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I36">
         <v>1</v>
@@ -2099,11 +2582,23 @@
       <c r="J36">
         <v>1</v>
       </c>
-      <c r="K36" t="s">
+      <c r="K36">
+        <v>1</v>
+      </c>
+      <c r="L36">
+        <v>1</v>
+      </c>
+      <c r="M36">
+        <v>1</v>
+      </c>
+      <c r="N36">
+        <v>1</v>
+      </c>
+      <c r="O36" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>109</v>
       </c>
@@ -2111,7 +2606,8 @@
         <v>110</v>
       </c>
       <c r="C37">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D37">
         <v>1</v>
@@ -2134,11 +2630,23 @@
       <c r="J37">
         <v>1</v>
       </c>
-      <c r="K37" t="s">
+      <c r="K37">
+        <v>1</v>
+      </c>
+      <c r="L37">
+        <v>1</v>
+      </c>
+      <c r="M37">
+        <v>1</v>
+      </c>
+      <c r="N37">
+        <v>1</v>
+      </c>
+      <c r="O37" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>112</v>
       </c>
@@ -2146,7 +2654,8 @@
         <v>113</v>
       </c>
       <c r="C38">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D38">
         <v>1</v>
@@ -2169,11 +2678,23 @@
       <c r="J38">
         <v>1</v>
       </c>
-      <c r="K38" t="s">
+      <c r="K38">
+        <v>1</v>
+      </c>
+      <c r="L38">
+        <v>1</v>
+      </c>
+      <c r="M38">
+        <v>1</v>
+      </c>
+      <c r="N38">
+        <v>1</v>
+      </c>
+      <c r="O38" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>115</v>
       </c>
@@ -2181,6 +2702,7 @@
         <v>116</v>
       </c>
       <c r="C39">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="D39">
@@ -2196,7 +2718,7 @@
         <v>1</v>
       </c>
       <c r="H39">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I39">
         <v>1</v>
@@ -2204,11 +2726,23 @@
       <c r="J39">
         <v>1</v>
       </c>
-      <c r="K39" t="s">
+      <c r="K39">
+        <v>1</v>
+      </c>
+      <c r="L39">
+        <v>1</v>
+      </c>
+      <c r="M39">
+        <v>1</v>
+      </c>
+      <c r="N39">
+        <v>1</v>
+      </c>
+      <c r="O39" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>118</v>
       </c>
@@ -2216,10 +2750,11 @@
         <v>119</v>
       </c>
       <c r="C40">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D40">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E40">
         <v>1</v>
@@ -2239,11 +2774,23 @@
       <c r="J40">
         <v>1</v>
       </c>
-      <c r="K40" t="s">
+      <c r="K40">
+        <v>1</v>
+      </c>
+      <c r="L40">
+        <v>1</v>
+      </c>
+      <c r="M40">
+        <v>1</v>
+      </c>
+      <c r="N40">
+        <v>1</v>
+      </c>
+      <c r="O40" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>121</v>
       </c>
@@ -2251,7 +2798,8 @@
         <v>122</v>
       </c>
       <c r="C41">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>2</v>
       </c>
       <c r="D41">
         <v>1</v>
@@ -2260,13 +2808,13 @@
         <v>1</v>
       </c>
       <c r="F41">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G41">
         <v>1</v>
       </c>
       <c r="H41">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I41">
         <v>1</v>
@@ -2274,11 +2822,23 @@
       <c r="J41">
         <v>1</v>
       </c>
-      <c r="K41" t="s">
+      <c r="K41">
+        <v>1</v>
+      </c>
+      <c r="L41">
+        <v>1</v>
+      </c>
+      <c r="M41">
+        <v>1</v>
+      </c>
+      <c r="N41">
+        <v>1</v>
+      </c>
+      <c r="O41" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>124</v>
       </c>
@@ -2286,10 +2846,11 @@
         <v>125</v>
       </c>
       <c r="C42">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D42">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E42">
         <v>1</v>
@@ -2309,11 +2870,23 @@
       <c r="J42">
         <v>1</v>
       </c>
-      <c r="K42" t="s">
+      <c r="K42">
+        <v>1</v>
+      </c>
+      <c r="L42">
+        <v>1</v>
+      </c>
+      <c r="M42">
+        <v>1</v>
+      </c>
+      <c r="N42">
+        <v>1</v>
+      </c>
+      <c r="O42" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>127</v>
       </c>
@@ -2321,7 +2894,8 @@
         <v>128</v>
       </c>
       <c r="C43">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D43">
         <v>1</v>
@@ -2344,11 +2918,23 @@
       <c r="J43">
         <v>1</v>
       </c>
-      <c r="K43" t="s">
+      <c r="K43">
+        <v>1</v>
+      </c>
+      <c r="L43">
+        <v>1</v>
+      </c>
+      <c r="M43">
+        <v>1</v>
+      </c>
+      <c r="N43">
+        <v>1</v>
+      </c>
+      <c r="O43" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>130</v>
       </c>
@@ -2356,7 +2942,8 @@
         <v>131</v>
       </c>
       <c r="C44">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D44">
         <v>1</v>
@@ -2379,11 +2966,23 @@
       <c r="J44">
         <v>1</v>
       </c>
-      <c r="K44" t="s">
+      <c r="K44">
+        <v>1</v>
+      </c>
+      <c r="L44">
+        <v>1</v>
+      </c>
+      <c r="M44">
+        <v>1</v>
+      </c>
+      <c r="N44">
+        <v>1</v>
+      </c>
+      <c r="O44" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>133</v>
       </c>
@@ -2391,7 +2990,8 @@
         <v>134</v>
       </c>
       <c r="C45">
-        <v>1</v>
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="D45">
         <v>1</v>
@@ -2414,11 +3014,23 @@
       <c r="J45">
         <v>1</v>
       </c>
-      <c r="K45" t="s">
+      <c r="K45">
+        <v>1</v>
+      </c>
+      <c r="L45">
+        <v>1</v>
+      </c>
+      <c r="M45">
+        <v>1</v>
+      </c>
+      <c r="N45">
+        <v>1</v>
+      </c>
+      <c r="O45" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>136</v>
       </c>
@@ -2426,6 +3038,7 @@
         <v>137</v>
       </c>
       <c r="C46">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="D46">
@@ -2438,7 +3051,7 @@
         <v>1</v>
       </c>
       <c r="G46">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H46">
         <v>1</v>
@@ -2449,53 +3062,34 @@
       <c r="J46">
         <v>1</v>
       </c>
-      <c r="K46" t="s">
+      <c r="K46">
+        <v>1</v>
+      </c>
+      <c r="L46">
+        <v>1</v>
+      </c>
+      <c r="M46">
+        <v>1</v>
+      </c>
+      <c r="N46">
+        <v>1</v>
+      </c>
+      <c r="O46" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A47" t="s">
-        <v>139</v>
-      </c>
-      <c r="B47" t="s">
-        <v>140</v>
-      </c>
-      <c r="C47">
-        <v>0</v>
-      </c>
+    <row r="47" spans="1:15" x14ac:dyDescent="0.2">
       <c r="D47">
-        <v>1</v>
-      </c>
-      <c r="E47">
-        <v>1</v>
-      </c>
-      <c r="F47">
-        <v>1</v>
+        <f>SUM(D2:D46)</f>
+        <v>43</v>
       </c>
       <c r="G47">
-        <v>1</v>
-      </c>
-      <c r="H47">
-        <v>1</v>
-      </c>
-      <c r="I47">
-        <v>1</v>
-      </c>
-      <c r="J47">
-        <v>1</v>
-      </c>
-      <c r="K47" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="C48">
-        <f>SUM(C2:C47)</f>
+        <f>SUM(G2:G46)</f>
         <v>43</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="C1:C48" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="G1:G47" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>